<commit_message>
Add qlXlOilVersion(.) function and tests
</commit_message>
<xml_diff>
--- a/tests/workbooktests/workbooks/test_quantlib.xlsx
+++ b/tests/workbooktests/workbooks/test_quantlib.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebastian\01_GitHub\sschlenkrich\QuantLibXlOil\tests\workbooktests\workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06EA5664-313C-40BB-A3E1-6BC096BE1A0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B6B3B26-9E63-4487-A4C0-AFE3E9649E9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3450" yWindow="-18675" windowWidth="30690" windowHeight="16530" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4020" yWindow="-18615" windowWidth="30690" windowHeight="16530" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -58,6 +58,23 @@
     </bk>
   </cellMetadata>
 </metadata>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+  <si>
+    <t>qlVersion</t>
+  </si>
+  <si>
+    <t>qlHexVersion</t>
+  </si>
+  <si>
+    <t>qlXlOilVersion</t>
+  </si>
+  <si>
+    <t>xloVersion</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -373,22 +390,58 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.109375" customWidth="1"/>
+    <col min="1" max="1" width="17" customWidth="1"/>
+    <col min="2" max="2" width="11.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" t="e" cm="1">
-        <f t="array" aca="1" ref="A1" ca="1">_xll.qlVersion()</f>
-        <v>#VALUE!</v>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="str" cm="1">
+        <f t="array" ref="B1">_xll.qlVersion()</f>
+        <v>1.41</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" t="e" cm="1">
-        <f t="array" aca="1" ref="A2" ca="1">_xll.qlHexVersion()</f>
-        <v>#VALUE!</v>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" cm="1">
+        <f t="array" ref="B2">_xll.qlHexVersion()</f>
+        <v>21037296</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" t="str" cm="1">
+        <f t="array" ref="B4">_xll.qlXlOilVersion()</f>
+        <v>0.41.0rc1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="str" cm="1">
+        <f t="array" ref="B6:C7">_xll.xloVersion()</f>
+        <v>Version</v>
+      </c>
+      <c r="C6" t="str">
+        <v>0.22.1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B7" t="str">
+        <v>BuildDate</v>
+      </c>
+      <c r="C7" t="str">
+        <v>"May 10 2026"</v>
       </c>
     </row>
   </sheetData>

</xml_diff>